<commit_message>
Daily slate 2026-05-31 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-29.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-29.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="E3" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F3" t="n">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="G3" t="n">
-        <v>63.3</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="4">
@@ -561,13 +561,13 @@
         <v>32</v>
       </c>
       <c r="E5" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G5" t="n">
-        <v>59.4</v>
+        <v>53.1</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>15</v>
       </c>
       <c r="G6" t="n">
-        <v>34.8</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" t="n">
         <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>62.5</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>371</v>
+        <v>388</v>
       </c>
       <c r="E8" t="n">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F8" t="n">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="G8" t="n">
-        <v>34.2</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E9" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G9" t="n">
-        <v>48.6</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>440</v>
+        <v>469</v>
       </c>
       <c r="E10" t="n">
-        <v>281</v>
+        <v>296</v>
       </c>
       <c r="F10" t="n">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="G10" t="n">
-        <v>63.9</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>267</v>
+        <v>286</v>
       </c>
       <c r="E11" t="n">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="F11" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G11" t="n">
-        <v>57.3</v>
+        <v>58.4</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="E12" t="n">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="F12" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G12" t="n">
-        <v>53.9</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="E13" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F13" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="G13" t="n">
-        <v>45.1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="E14" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F14" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="G14" t="n">
-        <v>27.1</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>282</v>
+        <v>332</v>
       </c>
       <c r="E15" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F15" t="n">
-        <v>227</v>
+        <v>272</v>
       </c>
       <c r="G15" t="n">
-        <v>19.5</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="E16" t="n">
         <v>21</v>
       </c>
       <c r="F16" t="n">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="G16" t="n">
-        <v>12.8</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="17">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2146</v>
+        <v>2267</v>
       </c>
       <c r="E17" t="n">
-        <v>512</v>
+        <v>541</v>
       </c>
       <c r="F17" t="n">
-        <v>1634</v>
+        <v>1726</v>
       </c>
       <c r="G17" t="n">
         <v>23.9</v>
@@ -1106,28 +1106,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -1139,19 +1139,19 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="R2" t="n">
         <v>30.4</v>
@@ -1169,10 +1169,10 @@
         <v>4</v>
       </c>
       <c r="X2" t="n">
-        <v>14</v>
+        <v>14.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="Z2" t="n">
         <v>85.7</v>
@@ -1485,13 +1485,13 @@
         <v>23</v>
       </c>
       <c r="D6" t="n">
-        <v>73.90000000000001</v>
+        <v>87</v>
       </c>
       <c r="E6" t="n">
         <v>23</v>
       </c>
       <c r="F6" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="G6" t="n">
         <v>12</v>
@@ -1509,7 +1509,7 @@
         <v>11</v>
       </c>
       <c r="L6" t="n">
-        <v>38.7</v>
+        <v>40.3</v>
       </c>
       <c r="M6" t="n">
         <v>62</v>
@@ -1542,13 +1542,13 @@
         <v>37</v>
       </c>
       <c r="Z6" t="n">
-        <v>48.1</v>
+        <v>33.3</v>
       </c>
       <c r="AA6" t="n">
         <v>54</v>
       </c>
       <c r="AB6" t="n">
-        <v>63.6</v>
+        <v>45.5</v>
       </c>
       <c r="AC6" t="n">
         <v>11</v>
@@ -1567,52 +1567,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>63.9</v>
+        <v>63.1</v>
       </c>
       <c r="C7" t="n">
-        <v>440</v>
+        <v>469</v>
       </c>
       <c r="D7" t="n">
-        <v>57.3</v>
+        <v>58.4</v>
       </c>
       <c r="E7" t="n">
-        <v>267</v>
+        <v>286</v>
       </c>
       <c r="F7" t="n">
-        <v>53.9</v>
+        <v>60</v>
       </c>
       <c r="G7" t="n">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="H7" t="n">
-        <v>45.1</v>
+        <v>47</v>
       </c>
       <c r="I7" t="n">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="J7" t="n">
-        <v>27.1</v>
+        <v>28.6</v>
       </c>
       <c r="K7" t="n">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="L7" t="n">
-        <v>19.5</v>
+        <v>18.1</v>
       </c>
       <c r="M7" t="n">
-        <v>282</v>
+        <v>332</v>
       </c>
       <c r="N7" t="n">
-        <v>12.8</v>
+        <v>12.1</v>
       </c>
       <c r="O7" t="n">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="P7" t="n">
         <v>23.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>2146</v>
+        <v>2267</v>
       </c>
       <c r="R7" t="n">
         <v>38.5</v>
@@ -1627,40 +1627,40 @@
         <v>11</v>
       </c>
       <c r="V7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="W7" t="n">
+        <v>24</v>
+      </c>
+      <c r="X7" t="n">
         <v>34.8</v>
       </c>
-      <c r="W7" t="n">
-        <v>23</v>
-      </c>
-      <c r="X7" t="n">
-        <v>34.2</v>
-      </c>
       <c r="Y7" t="n">
-        <v>371</v>
+        <v>388</v>
       </c>
       <c r="Z7" t="n">
-        <v>63.3</v>
+        <v>59.2</v>
       </c>
       <c r="AA7" t="n">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="AB7" t="n">
-        <v>59.4</v>
+        <v>53.1</v>
       </c>
       <c r="AC7" t="n">
         <v>32</v>
       </c>
       <c r="AD7" t="n">
-        <v>62.5</v>
+        <v>64</v>
       </c>
       <c r="AE7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AF7" t="n">
-        <v>48.6</v>
+        <v>51.2</v>
       </c>
       <c r="AG7" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>